<commit_message>
doc(Rapport, digramme uml, journal de travaille): mis à jour du JDT, ajout du diagramme UML et complétion du rapport
</commit_message>
<xml_diff>
--- a/Doc/T-P_POO-gillhorset-JournalTravail.xlsx
+++ b/Doc/T-P_POO-gillhorset-JournalTravail.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I-320\Projet\Local Repo\Doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\I-320\Projet\Local Repo\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCE5363-7B43-4786-9B17-BD4D16C79391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA20F15-2D77-4DF8-8426-CC090B5676DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6675" yWindow="1410" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="8835" yWindow="2490" windowWidth="27240" windowHeight="12750" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="93">
   <si>
     <t>Auteur:</t>
   </si>
@@ -317,6 +317,9 @@
   </si>
   <si>
     <t>Conseption du rapport</t>
+  </si>
+  <si>
+    <t>Rapport</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1336,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>235</c:v>
+                  <c:v>475</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1400,6 +1403,7 @@
     </c:legend>
     <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1407,7 +1411,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1773,6 +1776,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1780,7 +1784,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2257,16 +2260,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.17062937062937064</c:v>
+                  <c:v>0.15989515072083879</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.76363636363636367</c:v>
+                  <c:v>0.7155963302752294</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.5734265734265732E-2</c:v>
+                  <c:v>0.12450851900393185</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2424,6 +2427,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2431,7 +2435,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4504,7 +4507,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>59 heures 35 minutes</v>
+        <v>63 heures 35 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4519,7 +4522,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>2160</v>
+        <v>2400</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4527,7 +4530,7 @@
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>3575</v>
+        <v>3815</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5759,27 +5762,47 @@
       <c r="G59" s="40"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="62" t="str">
+      <c r="A60" s="62">
         <f>IF(ISBLANK(B60),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B60))</f>
-        <v/>
-      </c>
-      <c r="B60" s="30"/>
-      <c r="C60" s="31"/>
-      <c r="D60" s="32"/>
-      <c r="E60" s="33"/>
-      <c r="F60" s="39"/>
+        <v>44</v>
+      </c>
+      <c r="B60" s="30">
+        <v>45961</v>
+      </c>
+      <c r="C60" s="31">
+        <v>1</v>
+      </c>
+      <c r="D60" s="32">
+        <v>0</v>
+      </c>
+      <c r="E60" s="33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F60" s="39" t="s">
+        <v>92</v>
+      </c>
       <c r="G60" s="39"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="63" t="str">
+      <c r="A61" s="63">
         <f>IF(ISBLANK(B61),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B61))</f>
-        <v/>
-      </c>
-      <c r="B61" s="34"/>
-      <c r="C61" s="35"/>
-      <c r="D61" s="36"/>
-      <c r="E61" s="37"/>
-      <c r="F61" s="40"/>
+        <v>44</v>
+      </c>
+      <c r="B61" s="34">
+        <v>45962</v>
+      </c>
+      <c r="C61" s="35">
+        <v>3</v>
+      </c>
+      <c r="D61" s="36">
+        <v>0</v>
+      </c>
+      <c r="E61" s="37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F61" s="40" t="s">
+        <v>92</v>
+      </c>
       <c r="G61" s="40"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
@@ -11588,7 +11611,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.17062937062937064</v>
+        <v>0.15989515072083879</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11625,7 +11648,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.76363636363636367</v>
+        <v>0.7155963302752294</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11679,7 +11702,7 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>360</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
@@ -11687,7 +11710,7 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>235</v>
+        <v>475</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11695,11 +11718,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 55 min</v>
+        <v>7 h 55 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>6.5734265734265732E-2</v>
+        <v>0.12450851900393185</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11751,7 +11774,7 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>2160</v>
+        <v>2400</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
@@ -11759,18 +11782,18 @@
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>3575</v>
+        <v>3815</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>18</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>59 h 35 min</v>
+        <v>63 h 35 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.67708333333333337</v>
+        <v>0.72253787878787878</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>18</v>
@@ -11809,6 +11832,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11818,15 +11850,6 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12043,6 +12066,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -12051,14 +12082,6 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
doc(JDT): mise à jour du JDT
</commit_message>
<xml_diff>
--- a/Doc/T-P_POO-gillhorset-JournalTravail.xlsx
+++ b/Doc/T-P_POO-gillhorset-JournalTravail.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\I-320\Projet\Local Repo\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAA20F15-2D77-4DF8-8426-CC090B5676DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849F7E2D-6FBF-43E8-8175-449EEA5F7ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8835" yWindow="2490" windowWidth="27240" windowHeight="12750" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="20805" yWindow="2670" windowWidth="27240" windowHeight="12750" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -11506,7 +11506,10 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="49" orientation="landscape" r:id="rId1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="61" max="16383" man="1"/>
+  </rowBreaks>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
@@ -11832,27 +11835,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010080C9F2488912074FB587B9AD9ADAE5BB" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="020ab319e6f8d23aec07c29d6516d4ba">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xmlns:ns3="eefa3612-053e-497a-ae76-8a76877f5e22" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e15d3f914bf2a775f9387e5284d9197" ns2:_="" ns3:_="">
     <xsd:import namespace="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
@@ -12065,10 +12047,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D0F46EE-7556-4EFA-A1F5-7D69AEAE0E38}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -12087,20 +12101,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D0F46EE-7556-4EFA-A1F5-7D69AEAE0E38}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-    <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>